<commit_message>
Last game round 1
</commit_message>
<xml_diff>
--- a/Tournament_6_Teams.xlsx
+++ b/Tournament_6_Teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdulaziz\Desktop\Tournament\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA1C6FE-C479-4F4A-B895-4C26F16A9C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FD8E29-B8AB-481C-9ECE-17F3B6560735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -752,14 +752,18 @@
       <c r="C7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
+      <c r="D7" s="8">
+        <v>4</v>
+      </c>
+      <c r="E7" s="8">
+        <v>3</v>
+      </c>
       <c r="F7" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="8" t="str">
         <f t="array" ref="G7">_xlfn.IFS(AND(D7="", E7=""), "Have not started", OR(D7="", E7=""), "...", TRUE, "Finished")</f>
-        <v>Have not started</v>
+        <v>Finished</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
ROUND 2 GAME 1
</commit_message>
<xml_diff>
--- a/Tournament_6_Teams.xlsx
+++ b/Tournament_6_Teams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdulaziz\Desktop\Tournament\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\My_Tournament\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FD8E29-B8AB-481C-9ECE-17F3B6560735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5076E546-A298-471D-AD5A-E5DB7C33F35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matches" sheetId="1" r:id="rId1"/>
@@ -588,18 +588,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.36328125" style="5" customWidth="1"/>
-    <col min="4" max="5" width="8.7265625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.36328125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="8.7109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" style="9" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -622,7 +622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11">
         <v>1</v>
       </c>
@@ -646,7 +646,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -670,7 +670,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
         <v>1</v>
       </c>
@@ -694,7 +694,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>1</v>
       </c>
@@ -718,7 +718,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
         <v>1</v>
       </c>
@@ -742,7 +742,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
         <v>1</v>
       </c>
@@ -766,7 +766,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>2</v>
       </c>
@@ -776,17 +776,21 @@
       <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
+      <c r="D8" s="8">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8">
+        <v>7</v>
+      </c>
       <c r="F8" s="8" t="s">
         <v>14</v>
       </c>
       <c r="G8" s="8" t="str">
         <f t="array" ref="G8">_xlfn.IFS(AND(D8="", E8=""), "Have not started", OR(D8="", E8=""), "...", TRUE, "Finished")</f>
-        <v>Have not started</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>Finished</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>2</v>
       </c>
@@ -806,7 +810,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>2</v>
       </c>
@@ -826,7 +830,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
         <v>2</v>
       </c>
@@ -846,7 +850,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>2</v>
       </c>
@@ -866,7 +870,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>2</v>
       </c>
@@ -886,7 +890,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>3</v>
       </c>
@@ -906,7 +910,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
         <v>3</v>
       </c>
@@ -926,7 +930,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>3</v>
       </c>
@@ -946,7 +950,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>3</v>
       </c>
@@ -966,7 +970,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>3</v>
       </c>
@@ -986,7 +990,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>3</v>
       </c>
@@ -1006,7 +1010,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>4</v>
       </c>
@@ -1026,7 +1030,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>4</v>
       </c>
@@ -1046,7 +1050,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>4</v>
       </c>
@@ -1066,7 +1070,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>4</v>
       </c>
@@ -1086,7 +1090,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>4</v>
       </c>
@@ -1106,7 +1110,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>4</v>
       </c>
@@ -1126,7 +1130,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>5</v>
       </c>
@@ -1146,7 +1150,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>5</v>
       </c>
@@ -1166,7 +1170,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
         <v>5</v>
       </c>
@@ -1186,7 +1190,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>5</v>
       </c>
@@ -1206,7 +1210,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11">
         <v>5</v>
       </c>
@@ -1226,7 +1230,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
         <v>5</v>
       </c>
@@ -1255,9 +1259,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:J8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
@@ -1289,7 +1293,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1321,7 +1325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1353,7 +1357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1385,7 +1389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1417,7 +1421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1449,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1489,9 +1493,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:J8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
@@ -1523,7 +1527,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1555,7 +1559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1587,7 +1591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1619,7 +1623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1651,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1683,7 +1687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
ROUND 2 GAME 2
</commit_message>
<xml_diff>
--- a/Tournament_6_Teams.xlsx
+++ b/Tournament_6_Teams.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\My_Tournament\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5076E546-A298-471D-AD5A-E5DB7C33F35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FA96E1-57E0-41D8-9DCB-C248455F573C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -800,14 +800,18 @@
       <c r="C9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
+      <c r="D9" s="8">
+        <v>6</v>
+      </c>
+      <c r="E9" s="8">
+        <v>6</v>
+      </c>
       <c r="F9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="G9" s="8" t="str">
         <f t="array" ref="G9">_xlfn.IFS(AND(D9="", E9=""), "Have not started", OR(D9="", E9=""), "...", TRUE, "Finished")</f>
-        <v>Have not started</v>
+        <v>Finished</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Round 2 Game 3
</commit_message>
<xml_diff>
--- a/Tournament_6_Teams.xlsx
+++ b/Tournament_6_Teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\My_Tournament\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FA96E1-57E0-41D8-9DCB-C248455F573C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF93773E-4FA2-477E-AD20-4D292024D7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -824,14 +824,18 @@
       <c r="C10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="D10" s="8">
+        <v>7</v>
+      </c>
+      <c r="E10" s="8">
+        <v>7</v>
+      </c>
       <c r="F10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="G10" s="8" t="str">
         <f t="array" ref="G10">_xlfn.IFS(AND(D10="", E10=""), "Have not started", OR(D10="", E10=""), "...", TRUE, "Finished")</f>
-        <v>Have not started</v>
+        <v>Finished</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ROUND 2 GAME 4
</commit_message>
<xml_diff>
--- a/Tournament_6_Teams.xlsx
+++ b/Tournament_6_Teams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\My_Tournament\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdulaziz\Desktop\Tournament\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF93773E-4FA2-477E-AD20-4D292024D7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{711198C2-7248-445D-B936-0F23C5DCDBEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matches" sheetId="1" r:id="rId1"/>
@@ -588,18 +588,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="5" customWidth="1"/>
-    <col min="4" max="5" width="8.7109375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="8.7265625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" style="9" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -622,7 +622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11">
         <v>1</v>
       </c>
@@ -646,7 +646,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -670,7 +670,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11">
         <v>1</v>
       </c>
@@ -694,7 +694,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11">
         <v>1</v>
       </c>
@@ -718,7 +718,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11">
         <v>1</v>
       </c>
@@ -742,7 +742,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
         <v>1</v>
       </c>
@@ -766,7 +766,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11">
         <v>2</v>
       </c>
@@ -790,7 +790,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
         <v>2</v>
       </c>
@@ -814,7 +814,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11">
         <v>2</v>
       </c>
@@ -838,7 +838,7 @@
         <v>Finished</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
         <v>2</v>
       </c>
@@ -848,17 +848,21 @@
       <c r="C11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+      <c r="D11" s="8">
+        <v>5</v>
+      </c>
+      <c r="E11" s="8">
+        <v>7</v>
+      </c>
       <c r="F11" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G11" s="8" t="str">
         <f t="array" ref="G11">_xlfn.IFS(AND(D11="", E11=""), "Have not started", OR(D11="", E11=""), "...", TRUE, "Finished")</f>
-        <v>Have not started</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>Finished</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11">
         <v>2</v>
       </c>
@@ -878,7 +882,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
         <v>2</v>
       </c>
@@ -898,7 +902,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11">
         <v>3</v>
       </c>
@@ -918,7 +922,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11">
         <v>3</v>
       </c>
@@ -938,7 +942,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11">
         <v>3</v>
       </c>
@@ -958,7 +962,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11">
         <v>3</v>
       </c>
@@ -978,7 +982,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
         <v>3</v>
       </c>
@@ -998,7 +1002,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="11">
         <v>3</v>
       </c>
@@ -1018,7 +1022,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
         <v>4</v>
       </c>
@@ -1038,7 +1042,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
         <v>4</v>
       </c>
@@ -1058,7 +1062,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
         <v>4</v>
       </c>
@@ -1078,7 +1082,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
         <v>4</v>
       </c>
@@ -1098,7 +1102,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
         <v>4</v>
       </c>
@@ -1118,7 +1122,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
         <v>4</v>
       </c>
@@ -1138,7 +1142,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
         <v>5</v>
       </c>
@@ -1158,7 +1162,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
         <v>5</v>
       </c>
@@ -1178,7 +1182,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11">
         <v>5</v>
       </c>
@@ -1198,7 +1202,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
         <v>5</v>
       </c>
@@ -1218,7 +1222,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="11">
         <v>5</v>
       </c>
@@ -1238,7 +1242,7 @@
         <v>Have not started</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
         <v>5</v>
       </c>
@@ -1267,9 +1271,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:J8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
@@ -1301,7 +1305,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1333,7 +1337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1365,7 +1369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1397,7 +1401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1429,7 +1433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1461,7 +1465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1501,9 +1505,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:J8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
@@ -1535,7 +1539,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1567,7 +1571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1599,7 +1603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1631,7 +1635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1663,7 +1667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1695,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>

</xml_diff>